<commit_message>
Corrige le modele de perte de masse passive (Mm/Ml de la feuille Excel)
- Excel: ajoute Mm/minimumMass (=2, deja notre floor) et Ml/massLoose
  (2% au-dessus de 100, 1% en-dessous de 100, par 5s)
- config.ts: decay.threshold remplace la dependance implicite a player.startMass
- vanilla.json et folie.json: threshold=100, taux 2%/5s et 1%/5s (etaient
  1%/5s et 1%/10s calques sur M0)
- Point signale a l'utilisateur (non tranche): Folie demarre a 200, deja au-dessus
  du seuil litteral de 100 - decroit donc toujours au taux rapide
- metriques.md v0.4, 74 tests passants
</commit_message>
<xml_diff>
--- a/Angul.io - Master Sheet Engine & Documentation Technique.xlsx
+++ b/Angul.io - Master Sheet Engine & Documentation Technique.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z980"/>
+  <dimension ref="A1:Z982"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="82.38" customWidth="1" style="7" min="1" max="1"/>
@@ -1457,200 +1457,184 @@
       <c r="Z21" s="4" t="n"/>
     </row>
     <row r="22" ht="23.25" customHeight="1" s="7">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="n"/>
-      <c r="M22" s="4" t="n"/>
-      <c r="N22" s="4" t="n"/>
-      <c r="O22" s="4" t="n"/>
-      <c r="P22" s="4" t="n"/>
-      <c r="Q22" s="4" t="n"/>
-      <c r="R22" s="4" t="n"/>
-      <c r="S22" s="4" t="n"/>
-      <c r="T22" s="4" t="n"/>
-      <c r="U22" s="4" t="n"/>
-      <c r="V22" s="4" t="n"/>
-      <c r="W22" s="4" t="n"/>
-      <c r="X22" s="4" t="n"/>
-      <c r="Y22" s="4" t="n"/>
-      <c r="Z22" s="4" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mm</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>minimumMass</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Joueur</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Masse Minimum</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Masse minimum que le joueur atteint au fil du temps sans ingérer de masse</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Masse (uint)</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23" ht="23.25" customHeight="1" s="7">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ml</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>massLoose</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Joueur</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Perte de Masse</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Perte de la masse au fil du temps</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>% de la masse par 5 s</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2% au-dessus de 100, 1% en-dessous de 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="23.25" customHeight="1" s="7">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="n"/>
+      <c r="O24" s="4" t="n"/>
+      <c r="P24" s="4" t="n"/>
+      <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="n"/>
+      <c r="T24" s="4" t="n"/>
+      <c r="U24" s="4" t="n"/>
+      <c r="V24" s="4" t="n"/>
+      <c r="W24" s="4" t="n"/>
+      <c r="X24" s="4" t="n"/>
+      <c r="Y24" s="4" t="n"/>
+      <c r="Z24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="23.25" customHeight="1" s="7">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>2. MATRICE DE CONFIGURATION DES MODS DE JEU</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="n"/>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="n"/>
-      <c r="U23" s="2" t="n"/>
-      <c r="V23" s="2" t="n"/>
-      <c r="W23" s="2" t="n"/>
-      <c r="X23" s="2" t="n"/>
-      <c r="Y23" s="2" t="n"/>
-      <c r="Z23" s="2" t="n"/>
-    </row>
-    <row r="24" ht="23.25" customHeight="1" s="7">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2" t="n"/>
+      <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="2" t="n"/>
+      <c r="R25" s="2" t="n"/>
+      <c r="S25" s="2" t="n"/>
+      <c r="T25" s="2" t="n"/>
+      <c r="U25" s="2" t="n"/>
+      <c r="V25" s="2" t="n"/>
+      <c r="W25" s="2" t="n"/>
+      <c r="X25" s="2" t="n"/>
+      <c r="Y25" s="2" t="n"/>
+      <c r="Z25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="23.25" customHeight="1" s="7">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Catégorie</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Code ID / Paramètre</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Formule Mathématique</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Vanilla</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Folie</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="n"/>
-      <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
-      <c r="Q24" s="2" t="n"/>
-      <c r="R24" s="2" t="n"/>
-      <c r="S24" s="2" t="n"/>
-      <c r="T24" s="2" t="n"/>
-      <c r="U24" s="2" t="n"/>
-      <c r="V24" s="2" t="n"/>
-      <c r="W24" s="2" t="n"/>
-      <c r="X24" s="2" t="n"/>
-      <c r="Y24" s="2" t="n"/>
-      <c r="Z24" s="2" t="n"/>
-    </row>
-    <row r="25" ht="23.25" customHeight="1" s="7">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Joueur</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>startMass</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>M0</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
-      <c r="I25" s="4" t="n"/>
-      <c r="J25" s="4" t="n"/>
-      <c r="K25" s="4" t="n"/>
-      <c r="L25" s="4" t="n"/>
-      <c r="M25" s="4" t="n"/>
-      <c r="N25" s="4" t="n"/>
-      <c r="O25" s="4" t="n"/>
-      <c r="P25" s="4" t="n"/>
-      <c r="Q25" s="4" t="n"/>
-      <c r="R25" s="4" t="n"/>
-      <c r="S25" s="4" t="n"/>
-      <c r="T25" s="4" t="n"/>
-      <c r="U25" s="4" t="n"/>
-      <c r="V25" s="4" t="n"/>
-      <c r="W25" s="4" t="n"/>
-      <c r="X25" s="4" t="n"/>
-      <c r="Y25" s="4" t="n"/>
-      <c r="Z25" s="4" t="n"/>
-    </row>
-    <row r="26" ht="23.25" customHeight="1" s="7">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Joueur</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>maxSplits</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Smax</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
-      <c r="O26" s="4" t="n"/>
-      <c r="P26" s="4" t="n"/>
-      <c r="Q26" s="4" t="n"/>
-      <c r="R26" s="4" t="n"/>
-      <c r="S26" s="4" t="n"/>
-      <c r="T26" s="4" t="n"/>
-      <c r="U26" s="4" t="n"/>
-      <c r="V26" s="4" t="n"/>
-      <c r="W26" s="4" t="n"/>
-      <c r="X26" s="4" t="n"/>
-      <c r="Y26" s="4" t="n"/>
-      <c r="Z26" s="4" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2" t="n"/>
+      <c r="P26" s="2" t="n"/>
+      <c r="Q26" s="2" t="n"/>
+      <c r="R26" s="2" t="n"/>
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="n"/>
+      <c r="U26" s="2" t="n"/>
+      <c r="V26" s="2" t="n"/>
+      <c r="W26" s="2" t="n"/>
+      <c r="X26" s="2" t="n"/>
+      <c r="Y26" s="2" t="n"/>
+      <c r="Z26" s="2" t="n"/>
     </row>
     <row r="27" ht="23.25" customHeight="1" s="7">
       <c r="A27" s="4" t="inlineStr">
@@ -1660,23 +1644,19 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>recombineFormula</t>
+          <t>startMass</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>T_refusion(M) = Tbase + gamma_rec * M</t>
+          <t>M0</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>30 s (fixe)</t>
-        </is>
+      <c r="D27" s="4" t="n">
+        <v>50</v>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>15 s (fixe)</t>
-        </is>
+      <c r="E27" s="4" t="n">
+        <v>200</v>
       </c>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
@@ -1708,24 +1688,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>speedMultiplier</t>
+          <t>maxSplits</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>kv</t>
+          <t>Smax</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="D28" s="4" t="n">
+        <v>16</v>
       </c>
-      <c r="E28" s="8" t="n">
-        <v>2.5</v>
+      <c r="E28" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="F28" s="4" t="n"/>
-      <c r="G28" s="5" t="n"/>
+      <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
@@ -1754,22 +1732,26 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>ejectEfficiency</t>
+          <t>recombineFormula</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>eta_W = M_proj / M_cout</t>
+          <t>T_refusion(M) = Tbase + gamma_rec * M</t>
         </is>
       </c>
-      <c r="D29" s="6" t="n">
-        <v>1</v>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>30 s (fixe)</t>
+        </is>
       </c>
-      <c r="E29" s="6" t="n">
-        <v>1.2</v>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>15 s (fixe)</t>
+        </is>
       </c>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="4" t="n"/>
@@ -1793,31 +1775,29 @@
     <row r="30" ht="23.25" customHeight="1" s="7">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Arène</t>
+          <t>Joueur</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>arenaSize</t>
+          <t>speedMultiplier</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Wmap x Hmap</t>
+          <t>kv</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>15000 x 15000</t>
+          <t>1.0</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>20000 x 20000</t>
-        </is>
+      <c r="E30" s="8" t="n">
+        <v>2.5</v>
       </c>
       <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
+      <c r="G30" s="5" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="n"/>
@@ -1841,31 +1821,27 @@
     <row r="31" ht="23.25" customHeight="1" s="7">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Arène</t>
+          <t>Joueur</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>borderType</t>
+          <t>ejectEfficiency</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Condition aux limites</t>
+          <t>eta_W = M_proj / M_cout</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Mur strict</t>
-        </is>
+      <c r="D31" s="6" t="n">
+        <v>1</v>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rebond élastique renvoyant 80% de ma vitesse </t>
-        </is>
+      <c r="E31" s="6" t="n">
+        <v>1.2</v>
       </c>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="n"/>
@@ -1889,27 +1865,27 @@
     <row r="32" ht="23.25" customHeight="1" s="7">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Nourriture</t>
+          <t>Arène</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>foodDensity</t>
+          <t>arenaSize</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>D_food = N_food / (A / 1000²)</t>
+          <t>Wmap x Hmap</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>15 / 1000px²</t>
+          <t>15000 x 15000</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>30 / 1000px²</t>
+          <t>20000 x 20000</t>
         </is>
       </c>
       <c r="F32" s="4" t="n"/>
@@ -1937,25 +1913,27 @@
     <row r="33" ht="23.25" customHeight="1" s="7">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Nourriture</t>
+          <t>Arène</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>foodMass</t>
+          <t>borderType</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>M_food</t>
+          <t>Condition aux limites</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
-        <v>1</v>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Mur strict</t>
+        </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>2 - 8 (variable), Distribution de N-1 supérieur par rapport à N+1 (plus de petits que de gros)</t>
+          <t xml:space="preserve">Rebond élastique renvoyant 80% de ma vitesse </t>
         </is>
       </c>
       <c r="F33" s="4" t="n"/>
@@ -1988,22 +1966,22 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>foodRespawnRate</t>
+          <t>foodDensity</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>R_food (Hz)</t>
+          <t>D_food = N_food / (A / 1000²)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>100 / s</t>
+          <t>15 / 1000px²</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>200 / s</t>
+          <t>30 / 1000px²</t>
         </is>
       </c>
       <c r="F34" s="4" t="n"/>
@@ -2029,11 +2007,29 @@
       <c r="Z34" s="4" t="n"/>
     </row>
     <row r="35" ht="23.25" customHeight="1" s="7">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nourriture</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>foodMass</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>M_food</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>2 - 8 (variable), Distribution de N-1 supérieur par rapport à N+1 (plus de petits que de gros)</t>
+        </is>
+      </c>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
       <c r="H35" s="4" t="n"/>
@@ -2057,11 +2053,31 @@
       <c r="Z35" s="4" t="n"/>
     </row>
     <row r="36" ht="23.25" customHeight="1" s="7">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nourriture</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>foodRespawnRate</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>R_food (Hz)</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>100 / s</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>200 / s</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
       <c r="H36" s="4" t="n"/>
@@ -28516,6 +28532,62 @@
       <c r="Y980" s="4" t="n"/>
       <c r="Z980" s="4" t="n"/>
     </row>
+    <row r="981">
+      <c r="A981" s="4" t="n"/>
+      <c r="B981" s="4" t="n"/>
+      <c r="C981" s="4" t="n"/>
+      <c r="D981" s="4" t="n"/>
+      <c r="E981" s="4" t="n"/>
+      <c r="F981" s="4" t="n"/>
+      <c r="G981" s="4" t="n"/>
+      <c r="H981" s="4" t="n"/>
+      <c r="I981" s="4" t="n"/>
+      <c r="J981" s="4" t="n"/>
+      <c r="K981" s="4" t="n"/>
+      <c r="L981" s="4" t="n"/>
+      <c r="M981" s="4" t="n"/>
+      <c r="N981" s="4" t="n"/>
+      <c r="O981" s="4" t="n"/>
+      <c r="P981" s="4" t="n"/>
+      <c r="Q981" s="4" t="n"/>
+      <c r="R981" s="4" t="n"/>
+      <c r="S981" s="4" t="n"/>
+      <c r="T981" s="4" t="n"/>
+      <c r="U981" s="4" t="n"/>
+      <c r="V981" s="4" t="n"/>
+      <c r="W981" s="4" t="n"/>
+      <c r="X981" s="4" t="n"/>
+      <c r="Y981" s="4" t="n"/>
+      <c r="Z981" s="4" t="n"/>
+    </row>
+    <row r="982">
+      <c r="A982" s="4" t="n"/>
+      <c r="B982" s="4" t="n"/>
+      <c r="C982" s="4" t="n"/>
+      <c r="D982" s="4" t="n"/>
+      <c r="E982" s="4" t="n"/>
+      <c r="F982" s="4" t="n"/>
+      <c r="G982" s="4" t="n"/>
+      <c r="H982" s="4" t="n"/>
+      <c r="I982" s="4" t="n"/>
+      <c r="J982" s="4" t="n"/>
+      <c r="K982" s="4" t="n"/>
+      <c r="L982" s="4" t="n"/>
+      <c r="M982" s="4" t="n"/>
+      <c r="N982" s="4" t="n"/>
+      <c r="O982" s="4" t="n"/>
+      <c r="P982" s="4" t="n"/>
+      <c r="Q982" s="4" t="n"/>
+      <c r="R982" s="4" t="n"/>
+      <c r="S982" s="4" t="n"/>
+      <c r="T982" s="4" t="n"/>
+      <c r="U982" s="4" t="n"/>
+      <c r="V982" s="4" t="n"/>
+      <c r="W982" s="4" t="n"/>
+      <c r="X982" s="4" t="n"/>
+      <c r="Y982" s="4" t="n"/>
+      <c r="Z982" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>